<commit_message>
Clean_data.py is been updated with following features... 1) Project folders fetch 2)Select 250 stocks 3)Rename columns 4) Keep required columns
</commit_message>
<xml_diff>
--- a/data/raw/Book1.xlsx
+++ b/data/raw/Book1.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Khushi\my trade\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9378FB1E-D2D4-4E28-82EC-343E14965070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09A9310-51CB-4E03-B2F6-30A5259C1B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{A1FA5CC5-E2C2-4F51-9BAE-3F5476477926}"/>
+    <workbookView xWindow="-210" yWindow="0" windowWidth="9750" windowHeight="10170" xr2:uid="{A1FA5CC5-E2C2-4F51-9BAE-3F5476477926}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$84</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="99">
   <si>
     <t>S No.</t>
   </si>
@@ -98,9 +101,6 @@
     <t>ICICI Prudential AMC</t>
   </si>
   <si>
-    <t>Return</t>
-  </si>
-  <si>
     <t>TECHM</t>
   </si>
   <si>
@@ -261,6 +261,81 @@
   </si>
   <si>
     <t>LAURUSLABS</t>
+  </si>
+  <si>
+    <t>Today's closing price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIPLA </t>
+  </si>
+  <si>
+    <t>MEDANTA</t>
+  </si>
+  <si>
+    <t>SYRMA</t>
+  </si>
+  <si>
+    <t>Vedanta Alum</t>
+  </si>
+  <si>
+    <t>Dixon Technologies</t>
+  </si>
+  <si>
+    <t>Gokaldas Exports</t>
+  </si>
+  <si>
+    <t>Gujarat Fluorochem</t>
+  </si>
+  <si>
+    <t>Genus Power</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Excepted Return</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> bharat forge</t>
+  </si>
+  <si>
+    <t>shriram finance</t>
+  </si>
+  <si>
+    <t>Hind petro</t>
+  </si>
+  <si>
+    <t>Axis Bank</t>
+  </si>
+  <si>
+    <t>welcorp</t>
+  </si>
+  <si>
+    <t>Maruti</t>
+  </si>
+  <si>
+    <t>ABCentral</t>
+  </si>
+  <si>
+    <t>JSW steel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Star Health </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max Health </t>
+  </si>
+  <si>
+    <t>kirloskar oli engines</t>
+  </si>
+  <si>
+    <t>Marico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Granules </t>
+  </si>
+  <si>
+    <t>Torrent Pharmaceuticals</t>
   </si>
 </sst>
 </file>
@@ -276,12 +351,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -296,11 +383,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -635,7 +724,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11702C7E-E6DA-4340-BEE9-A978C9B55E59}">
-  <dimension ref="A1:J82"/>
+  <dimension ref="A1:L131"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
@@ -644,13 +733,14 @@
     <col min="4" max="4" width="11.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.36328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.36328125" customWidth="1"/>
-    <col min="8" max="8" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.36328125" customWidth="1"/>
+    <col min="9" max="9" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -670,19 +760,25 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="H1" t="s">
+        <v>84</v>
+      </c>
+      <c r="I1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="L1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -701,8 +797,12 @@
       <c r="F2">
         <v>3450</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H2" s="2">
+        <f>(E2-D2)/D2</f>
+        <v>4.2962125494629737E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -715,8 +815,12 @@
       <c r="D3">
         <v>748</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H3" s="2">
+        <f t="shared" ref="H3:H27" si="0">(E3-D3)/D3</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -729,14 +833,18 @@
       <c r="D4">
         <v>2056</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+      <c r="I4" s="1">
         <v>46191</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>2365</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -752,14 +860,18 @@
       <c r="E5">
         <v>1160</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
+        <f t="shared" si="0"/>
+        <v>0.15308151093439365</v>
+      </c>
+      <c r="I5" s="1">
         <v>46175</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>1344</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -775,8 +887,12 @@
       <c r="E6">
         <v>6600</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H6" s="2">
+        <f t="shared" si="0"/>
+        <v>0.12225811936745451</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -795,14 +911,18 @@
       <c r="F7">
         <v>1438</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
+        <f t="shared" si="0"/>
+        <v>1.8543956043956044E-2</v>
+      </c>
+      <c r="I7" s="1">
         <v>46175</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>1488</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -818,8 +938,12 @@
       <c r="E8">
         <v>580</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H8" s="2">
+        <f t="shared" si="0"/>
+        <v>0.3200118345888619</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -835,8 +959,12 @@
       <c r="E9">
         <v>3850</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H9" s="2">
+        <f t="shared" si="0"/>
+        <v>0.23999948467553878</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -852,8 +980,12 @@
       <c r="E10">
         <v>1450</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H10" s="2">
+        <f t="shared" si="0"/>
+        <v>0.20000331035395966</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -869,8 +1001,12 @@
       <c r="E11">
         <v>1100</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H11" s="2">
+        <f t="shared" si="0"/>
+        <v>0.18000429092469422</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -886,13 +1022,17 @@
       <c r="E12">
         <v>3850</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H12" s="2">
+        <f t="shared" si="0"/>
+        <v>0.15999843324886945</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C13" s="1">
         <v>46175</v>
@@ -903,13 +1043,17 @@
       <c r="E13">
         <v>1720</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H13" s="2">
+        <f t="shared" si="0"/>
+        <v>0.11471160077770577</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C14" s="1">
         <v>46175</v>
@@ -917,13 +1061,17 @@
       <c r="D14">
         <v>434</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H14" s="2">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C15" s="1">
         <v>46175</v>
@@ -934,13 +1082,17 @@
       <c r="E15">
         <v>235</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H15" s="2">
+        <f t="shared" si="0"/>
+        <v>0.27027027027027029</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C16" s="1">
         <v>46175</v>
@@ -951,8 +1103,12 @@
       <c r="E16">
         <v>2050</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H16" s="2">
+        <f t="shared" si="0"/>
+        <v>0.14974761637689288</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -971,13 +1127,17 @@
       <c r="F17">
         <v>705</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H17" s="2">
+        <f t="shared" si="0"/>
+        <v>0.16036505867014342</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C18" s="1">
         <v>46176</v>
@@ -985,13 +1145,17 @@
       <c r="D18">
         <v>835</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H18" s="2">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C19" s="1">
         <v>46176</v>
@@ -1005,13 +1169,17 @@
       <c r="F19">
         <v>510</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H19" s="2">
+        <f t="shared" si="0"/>
+        <v>8.0074487895716945E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C20" s="1">
         <v>46176</v>
@@ -1019,13 +1187,17 @@
       <c r="D20">
         <v>1074</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H20" s="2">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C21" s="1">
         <v>46176</v>
@@ -1033,13 +1205,17 @@
       <c r="D21">
         <v>406</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H21" s="2">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C22" s="1">
         <v>46176</v>
@@ -1050,12 +1226,16 @@
       <c r="E22">
         <v>1200</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H22" s="2">
+        <f t="shared" si="0"/>
+        <v>0.10091743119266056</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C23" s="1">
@@ -1070,13 +1250,20 @@
       <c r="F23">
         <v>705</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="G23">
+        <v>1153</v>
+      </c>
+      <c r="H23" s="2">
+        <f t="shared" si="0"/>
+        <v>0.16036505867014342</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C24" s="1">
         <v>46177</v>
@@ -1090,13 +1277,17 @@
       <c r="F24">
         <v>2040</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H24" s="2">
+        <f t="shared" si="0"/>
+        <v>0.13476473275468251</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C25" s="1">
         <v>46182</v>
@@ -1110,19 +1301,23 @@
       <c r="F25">
         <v>295</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
+        <f t="shared" si="0"/>
+        <v>6.5573770491803282E-2</v>
+      </c>
+      <c r="I25" s="1">
         <v>46189</v>
       </c>
-      <c r="I25">
+      <c r="J25">
         <v>320</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C26" s="1">
         <v>46182</v>
@@ -1130,13 +1325,17 @@
       <c r="D26">
         <v>168.6</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H26" s="2">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C27" s="1">
         <v>46182</v>
@@ -1147,8 +1346,15 @@
       <c r="E27">
         <v>360</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H27" s="2">
+        <f t="shared" si="0"/>
+        <v>0.34328358208955223</v>
+      </c>
+      <c r="J27">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1167,19 +1373,19 @@
       <c r="F28">
         <v>705</v>
       </c>
-      <c r="H28" s="1">
+      <c r="I28" s="1">
         <v>46184</v>
       </c>
-      <c r="I28">
+      <c r="J28">
         <v>960</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C29" s="1">
         <v>46184</v>
@@ -1194,12 +1400,12 @@
         <v>1388</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C30" s="1">
         <v>46184</v>
@@ -1211,12 +1417,12 @@
         <v>1450</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C31" s="1">
         <v>46184</v>
@@ -1228,12 +1434,12 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C32" s="1">
         <v>46184</v>
@@ -1250,7 +1456,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C33" s="1">
         <v>46185</v>
@@ -1270,7 +1476,7 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C34" s="1">
         <v>46185</v>
@@ -1284,7 +1490,7 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C35" s="1">
         <v>46185</v>
@@ -1298,7 +1504,7 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C36" s="1">
         <v>46185</v>
@@ -1315,7 +1521,7 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C37" s="1">
         <v>46185</v>
@@ -1335,7 +1541,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C38" s="1">
         <v>46188</v>
@@ -1355,7 +1561,7 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C39" s="1">
         <v>46188</v>
@@ -1372,7 +1578,7 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C40" s="1">
         <v>46188</v>
@@ -1386,7 +1592,7 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C41" s="1">
         <v>46188</v>
@@ -1400,7 +1606,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C42" s="1">
         <v>46188</v>
@@ -1420,7 +1626,7 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C43" s="1">
         <v>46189</v>
@@ -1440,7 +1646,7 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C44" s="1">
         <v>46189</v>
@@ -1454,7 +1660,7 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C45" s="1">
         <v>46189</v>
@@ -1468,7 +1674,7 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C46" s="1">
         <v>46189</v>
@@ -1482,7 +1688,7 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C47" s="1">
         <v>46189</v>
@@ -1496,7 +1702,7 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C48" s="1">
         <v>46189</v>
@@ -1505,12 +1711,12 @@
         <v>125</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C49" s="1">
         <v>46189</v>
@@ -1519,12 +1725,12 @@
         <v>1765</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C50" s="1">
         <v>46189</v>
@@ -1532,22 +1738,22 @@
       <c r="D50">
         <v>210</v>
       </c>
-      <c r="G50" s="2">
+      <c r="H50" s="2">
         <v>1.4E-2</v>
       </c>
-      <c r="H50" s="1">
+      <c r="I50" s="1">
         <v>46189</v>
       </c>
-      <c r="I50">
+      <c r="J50">
         <v>218</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C51" s="1">
         <v>46189</v>
@@ -1562,12 +1768,12 @@
         <v>76</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C52" s="1">
         <v>46190</v>
@@ -1582,12 +1788,12 @@
         <v>1820</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C53" s="1">
         <v>46190</v>
@@ -1596,7 +1802,7 @@
         <v>1079</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>53</v>
       </c>
@@ -1613,12 +1819,12 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C55" s="1">
         <v>46190</v>
@@ -1627,12 +1833,12 @@
         <v>374</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C56" s="1">
         <v>46190</v>
@@ -1641,12 +1847,12 @@
         <v>1520</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C57" s="1">
         <v>46190</v>
@@ -1660,14 +1866,14 @@
       <c r="F57">
         <v>204</v>
       </c>
-      <c r="H57" s="1"/>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="I57" s="1"/>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C58" s="1">
         <v>46190</v>
@@ -1681,19 +1887,19 @@
       <c r="F58">
         <v>151</v>
       </c>
-      <c r="H58" s="1">
+      <c r="I58" s="1">
         <v>46190</v>
       </c>
-      <c r="I58">
+      <c r="J58">
         <v>156.6</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C59" s="1">
         <v>46191</v>
@@ -1705,7 +1911,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>59</v>
       </c>
@@ -1721,13 +1927,16 @@
       <c r="E60">
         <v>2600</v>
       </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J60">
+        <v>2450</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C61" s="1">
         <v>46191</v>
@@ -1736,12 +1945,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C62" s="1">
         <v>46191</v>
@@ -1750,12 +1959,12 @@
         <v>1026</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C63" s="1">
         <v>46191</v>
@@ -1764,12 +1973,12 @@
         <v>420</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C64" s="1">
         <v>46191</v>
@@ -1784,12 +1993,12 @@
         <v>930</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C65" s="1">
         <v>46192</v>
@@ -1804,12 +2013,12 @@
         <v>3415</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C66" s="1">
         <v>46192</v>
@@ -1821,12 +2030,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C67" s="1">
         <v>46192</v>
@@ -1838,12 +2047,12 @@
         <v>8450</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C68" s="1">
         <v>46192</v>
@@ -1852,12 +2061,12 @@
         <v>406</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C69" s="1">
         <v>46192</v>
@@ -1866,12 +2075,12 @@
         <v>1446</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C70" s="1">
         <v>46192</v>
@@ -1886,26 +2095,26 @@
         <v>2845</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C71" s="1">
         <v>46192</v>
       </c>
-      <c r="G71" s="3">
+      <c r="H71" s="3">
         <v>0.09</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C72" s="1">
         <v>46195</v>
@@ -1920,12 +2129,15 @@
         <v>3415</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>71</v>
+        <v>70</v>
+      </c>
+      <c r="C73" s="1">
+        <v>46195</v>
       </c>
       <c r="D73">
         <v>1992</v>
@@ -1933,69 +2145,84 @@
       <c r="E73">
         <v>2350</v>
       </c>
-      <c r="G73" s="3">
+      <c r="H73" s="3">
         <v>0.2</v>
       </c>
-      <c r="H73" s="1">
+      <c r="I73" s="1">
         <v>46195</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>73</v>
       </c>
       <c r="B74" t="s">
         <v>15</v>
       </c>
+      <c r="C74" s="1">
+        <v>46195</v>
+      </c>
       <c r="D74">
         <v>416</v>
       </c>
       <c r="E74">
         <v>580</v>
       </c>
-      <c r="G74" s="3">
+      <c r="H74" s="3">
         <v>0.05</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>72</v>
+        <v>71</v>
+      </c>
+      <c r="C75" s="1">
+        <v>46195</v>
       </c>
       <c r="D75">
         <v>1889</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>73</v>
+        <v>72</v>
+      </c>
+      <c r="C76" s="1">
+        <v>46195</v>
       </c>
       <c r="D76">
         <v>264</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>56</v>
+        <v>55</v>
+      </c>
+      <c r="C77" s="1">
+        <v>46195</v>
       </c>
       <c r="D77">
         <v>376</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>74</v>
+        <v>73</v>
+      </c>
+      <c r="C78" s="1">
+        <v>46195</v>
       </c>
       <c r="D78">
         <v>1413</v>
@@ -2007,27 +2234,634 @@
         <v>1340</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>78</v>
       </c>
-    </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B79" t="s">
+        <v>75</v>
+      </c>
+      <c r="C79" s="1">
+        <v>46196</v>
+      </c>
+      <c r="D79">
+        <v>1415</v>
+      </c>
+      <c r="E79">
+        <v>1530</v>
+      </c>
+      <c r="F79">
+        <v>1360</v>
+      </c>
+      <c r="I79" s="1">
+        <v>46203</v>
+      </c>
+      <c r="J79">
+        <v>1485</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>79</v>
       </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B80" t="s">
+        <v>47</v>
+      </c>
+      <c r="C80" s="1">
+        <v>46196</v>
+      </c>
+      <c r="D80">
+        <v>2103</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>80</v>
       </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B81" t="s">
+        <v>15</v>
+      </c>
+      <c r="C81" s="1">
+        <v>46196</v>
+      </c>
+      <c r="D81">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>81</v>
       </c>
+      <c r="B82" t="s">
+        <v>76</v>
+      </c>
+      <c r="C82" s="1">
+        <v>46196</v>
+      </c>
+      <c r="D82">
+        <v>1288</v>
+      </c>
+      <c r="E82">
+        <v>1490</v>
+      </c>
+      <c r="H82" s="3">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C83" s="1">
+        <v>46196</v>
+      </c>
+      <c r="D83">
+        <v>1336</v>
+      </c>
+      <c r="E83">
+        <v>1620</v>
+      </c>
+      <c r="H83" s="3">
+        <v>0.21</v>
+      </c>
+      <c r="J83">
+        <v>1430</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="s">
+        <v>63</v>
+      </c>
+      <c r="C84" s="1">
+        <v>46196</v>
+      </c>
+      <c r="D84">
+        <v>3653</v>
+      </c>
+      <c r="E84">
+        <v>4100</v>
+      </c>
+      <c r="F84">
+        <v>3415</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="s">
+        <v>78</v>
+      </c>
+      <c r="C85" s="1">
+        <v>46197</v>
+      </c>
+      <c r="D85">
+        <v>454</v>
+      </c>
+      <c r="E85">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86" t="s">
+        <v>79</v>
+      </c>
+      <c r="C86" s="1">
+        <v>46197</v>
+      </c>
+      <c r="D86">
+        <v>12667</v>
+      </c>
+      <c r="E86">
+        <v>15290</v>
+      </c>
+      <c r="F86">
+        <v>11400</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C87" s="1">
+        <v>46197</v>
+      </c>
+      <c r="D87">
+        <v>829</v>
+      </c>
+      <c r="E87">
+        <v>1110</v>
+      </c>
+      <c r="L87">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88" t="s">
+        <v>81</v>
+      </c>
+      <c r="C88" s="1">
+        <v>46197</v>
+      </c>
+      <c r="D88">
+        <v>3891</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89" t="s">
+        <v>82</v>
+      </c>
+      <c r="C89" s="1">
+        <v>46197</v>
+      </c>
+      <c r="D89">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C90" s="1">
+        <v>46197</v>
+      </c>
+      <c r="D90">
+        <v>1112</v>
+      </c>
+      <c r="E90">
+        <v>1185</v>
+      </c>
+      <c r="F90">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="91" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91" t="s">
+        <v>22</v>
+      </c>
+      <c r="C91" s="1">
+        <v>46197</v>
+      </c>
+      <c r="D91">
+        <v>199</v>
+      </c>
+      <c r="E91">
+        <v>204</v>
+      </c>
+      <c r="F91">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92" t="s">
+        <v>63</v>
+      </c>
+      <c r="C92" s="1">
+        <v>46198</v>
+      </c>
+      <c r="D92">
+        <v>3653</v>
+      </c>
+      <c r="E92">
+        <v>4100</v>
+      </c>
+      <c r="F92">
+        <v>3415</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="s">
+        <v>85</v>
+      </c>
+      <c r="C93" s="1">
+        <v>46198</v>
+      </c>
+      <c r="D93">
+        <v>2123</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94" t="s">
+        <v>86</v>
+      </c>
+      <c r="C94" s="1">
+        <v>46198</v>
+      </c>
+      <c r="D94">
+        <v>1019</v>
+      </c>
+      <c r="E94">
+        <v>1175</v>
+      </c>
+      <c r="G94">
+        <v>1033</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95" t="s">
+        <v>87</v>
+      </c>
+      <c r="C95" s="1">
+        <v>46198</v>
+      </c>
+      <c r="D95">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A96">
+        <v>95</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C96" s="1">
+        <v>46198</v>
+      </c>
+      <c r="D96">
+        <v>1384</v>
+      </c>
+      <c r="E96">
+        <v>1441</v>
+      </c>
+      <c r="F96">
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C97" s="1">
+        <v>46202</v>
+      </c>
+      <c r="D97">
+        <v>1455</v>
+      </c>
+      <c r="E97">
+        <v>1570</v>
+      </c>
+      <c r="F97">
+        <v>1380</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A98">
+        <v>97</v>
+      </c>
+      <c r="B98" t="s">
+        <v>90</v>
+      </c>
+      <c r="C98" s="1">
+        <v>46202</v>
+      </c>
+      <c r="D98">
+        <v>13735</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A99">
+        <v>98</v>
+      </c>
+      <c r="B99" t="s">
+        <v>91</v>
+      </c>
+      <c r="C99" s="1">
+        <v>46202</v>
+      </c>
+      <c r="D99">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A100">
+        <v>99</v>
+      </c>
+      <c r="B100" t="s">
+        <v>92</v>
+      </c>
+      <c r="C100" s="1">
+        <v>46202</v>
+      </c>
+      <c r="D100">
+        <v>1231</v>
+      </c>
+      <c r="E100">
+        <v>1520</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A101">
+        <v>100</v>
+      </c>
+      <c r="B101" t="s">
+        <v>93</v>
+      </c>
+      <c r="C101" s="1">
+        <v>46202</v>
+      </c>
+      <c r="D101">
+        <v>575</v>
+      </c>
+      <c r="E101">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A102">
+        <v>101</v>
+      </c>
+      <c r="B102" t="s">
+        <v>94</v>
+      </c>
+      <c r="C102" s="1">
+        <v>46202</v>
+      </c>
+      <c r="D102">
+        <v>1132</v>
+      </c>
+      <c r="E102">
+        <v>1329</v>
+      </c>
+      <c r="F102">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A103">
+        <v>102</v>
+      </c>
+      <c r="B103" t="s">
+        <v>86</v>
+      </c>
+      <c r="C103" s="1">
+        <v>46202</v>
+      </c>
+      <c r="D103">
+        <v>1046</v>
+      </c>
+      <c r="E103">
+        <v>1205</v>
+      </c>
+      <c r="F103">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A104">
+        <v>103</v>
+      </c>
+      <c r="B104" t="s">
+        <v>95</v>
+      </c>
+      <c r="D104">
+        <v>2441</v>
+      </c>
+      <c r="E104">
+        <v>2750</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A105">
+        <v>104</v>
+      </c>
+      <c r="B105" t="s">
+        <v>96</v>
+      </c>
+      <c r="D105">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A106">
+        <v>105</v>
+      </c>
+      <c r="B106" t="s">
+        <v>97</v>
+      </c>
+      <c r="D106">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A107">
+        <v>106</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D107">
+        <v>4628</v>
+      </c>
+      <c r="E107">
+        <v>4850</v>
+      </c>
+      <c r="F107">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A108">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A109">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A110">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A111">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A112">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A113">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A114">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A115">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A116">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A117">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A118">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A119">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A120">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A121">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A122">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A123">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A124">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A125">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A126">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A127">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A128">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A129">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A130">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A131">
+        <v>130</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K84" xr:uid="{11702C7E-E6DA-4340-BEE9-A978C9B55E59}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added folder feature_engineer and indicator file in data
</commit_message>
<xml_diff>
--- a/data/raw/Book1.xlsx
+++ b/data/raw/Book1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Khushi\my trade\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09A9310-51CB-4E03-B2F6-30A5259C1B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC81B6D7-3E67-4F6D-BD5E-669FE6738199}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-210" yWindow="0" windowWidth="9750" windowHeight="10170" xr2:uid="{A1FA5CC5-E2C2-4F51-9BAE-3F5476477926}"/>
+    <workbookView xWindow="-50" yWindow="0" windowWidth="9610" windowHeight="10170" xr2:uid="{A1FA5CC5-E2C2-4F51-9BAE-3F5476477926}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="108">
   <si>
     <t>S No.</t>
   </si>
@@ -336,6 +336,33 @@
   </si>
   <si>
     <t>Torrent Pharmaceuticals</t>
+  </si>
+  <si>
+    <t>Aditya Birla Real Estate</t>
+  </si>
+  <si>
+    <t>Credit access grameen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CGPOWER </t>
+  </si>
+  <si>
+    <t>Bajaj Finance</t>
+  </si>
+  <si>
+    <t>Naukri</t>
+  </si>
+  <si>
+    <t>Aether</t>
+  </si>
+  <si>
+    <t>ONGC</t>
+  </si>
+  <si>
+    <t>AADHAR HOUSING FINANCE</t>
+  </si>
+  <si>
+    <t>NYKAA</t>
   </si>
 </sst>
 </file>
@@ -728,8 +755,8 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.26953125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.36328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.08984375" bestFit="1" customWidth="1"/>
@@ -2693,6 +2720,9 @@
       <c r="B104" t="s">
         <v>95</v>
       </c>
+      <c r="C104" s="1">
+        <v>46204</v>
+      </c>
       <c r="D104">
         <v>2441</v>
       </c>
@@ -2707,6 +2737,9 @@
       <c r="B105" t="s">
         <v>96</v>
       </c>
+      <c r="C105" s="1">
+        <v>46204</v>
+      </c>
       <c r="D105">
         <v>840</v>
       </c>
@@ -2718,6 +2751,9 @@
       <c r="B106" t="s">
         <v>97</v>
       </c>
+      <c r="C106" s="1">
+        <v>46204</v>
+      </c>
       <c r="D106">
         <v>802</v>
       </c>
@@ -2729,6 +2765,9 @@
       <c r="B107" s="4" t="s">
         <v>98</v>
       </c>
+      <c r="C107" s="1">
+        <v>46204</v>
+      </c>
       <c r="D107">
         <v>4628</v>
       </c>
@@ -2743,103 +2782,265 @@
       <c r="A108">
         <v>107</v>
       </c>
+      <c r="B108" t="s">
+        <v>99</v>
+      </c>
+      <c r="C108" s="1">
+        <v>46205</v>
+      </c>
+      <c r="D108">
+        <v>1396</v>
+      </c>
+      <c r="E108">
+        <v>1940</v>
+      </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>108</v>
       </c>
+      <c r="B109" t="s">
+        <v>100</v>
+      </c>
+      <c r="C109" s="1">
+        <v>46205</v>
+      </c>
+      <c r="D109">
+        <v>1503</v>
+      </c>
+      <c r="E109">
+        <v>1780</v>
+      </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>109</v>
       </c>
+      <c r="B110" t="s">
+        <v>101</v>
+      </c>
+      <c r="C110" s="1">
+        <v>46205</v>
+      </c>
+      <c r="D110">
+        <v>976</v>
+      </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>110</v>
       </c>
+      <c r="B111" t="s">
+        <v>15</v>
+      </c>
+      <c r="C111" s="1">
+        <v>46205</v>
+      </c>
+      <c r="D111">
+        <v>508</v>
+      </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>111</v>
       </c>
-    </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B112" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C112" s="1">
+        <v>46205</v>
+      </c>
+      <c r="D112">
+        <v>1628</v>
+      </c>
+      <c r="E112">
+        <v>1760</v>
+      </c>
+      <c r="F112">
+        <v>1540</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>112</v>
       </c>
-    </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B113" t="s">
+        <v>99</v>
+      </c>
+      <c r="C113" s="1">
+        <v>46206</v>
+      </c>
+      <c r="D113">
+        <v>1412</v>
+      </c>
+      <c r="E113">
+        <v>1586</v>
+      </c>
+      <c r="F113">
+        <v>1331</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>113</v>
       </c>
-    </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B114" t="s">
+        <v>102</v>
+      </c>
+      <c r="C114" s="1">
+        <v>46206</v>
+      </c>
+      <c r="D114">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>114</v>
       </c>
-    </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B115" t="s">
+        <v>96</v>
+      </c>
+      <c r="C115" s="1">
+        <v>46206</v>
+      </c>
+      <c r="D115">
+        <v>856</v>
+      </c>
+      <c r="E115">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>115</v>
       </c>
-    </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B116" t="s">
+        <v>103</v>
+      </c>
+      <c r="C116" s="1">
+        <v>46206</v>
+      </c>
+      <c r="D116">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>116</v>
       </c>
-    </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B117" t="s">
+        <v>104</v>
+      </c>
+      <c r="C117" s="1">
+        <v>46206</v>
+      </c>
+      <c r="D117">
+        <v>1360</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>117</v>
       </c>
-    </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B118" t="s">
+        <v>23</v>
+      </c>
+      <c r="C118" s="1">
+        <v>46206</v>
+      </c>
+      <c r="D118">
+        <v>1882</v>
+      </c>
+      <c r="E118">
+        <v>2017</v>
+      </c>
+      <c r="F118">
+        <v>1810</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>118</v>
       </c>
-    </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B119" t="s">
+        <v>105</v>
+      </c>
+      <c r="C119" s="1">
+        <v>46209</v>
+      </c>
+      <c r="D119">
+        <v>235</v>
+      </c>
+      <c r="E119">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>119</v>
       </c>
-    </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B120" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C120" s="1">
+        <v>46209</v>
+      </c>
+      <c r="D120">
+        <v>548</v>
+      </c>
+      <c r="E120">
+        <v>612</v>
+      </c>
+      <c r="F120">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>120</v>
       </c>
-    </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B121" t="s">
+        <v>107</v>
+      </c>
+      <c r="C121" s="1">
+        <v>46209</v>
+      </c>
+      <c r="D121">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>121</v>
       </c>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>122</v>
       </c>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>123</v>
       </c>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>124</v>
       </c>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>125</v>
       </c>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>126</v>
       </c>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>127</v>
       </c>

</xml_diff>

<commit_message>
Update fetching of data to get all data instead of just top 250 rows
</commit_message>
<xml_diff>
--- a/data/raw/Book1.xlsx
+++ b/data/raw/Book1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Khushi\my trade\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE7D081D-0343-4D2E-8276-578E354BBF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDAE28C3-2E2D-4C18-A7E1-2C3E9A89475F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11430" yWindow="0" windowWidth="7860" windowHeight="10170" xr2:uid="{A1FA5CC5-E2C2-4F51-9BAE-3F5476477926}"/>
+    <workbookView xWindow="11500" yWindow="0" windowWidth="7550" windowHeight="10170" xr2:uid="{A1FA5CC5-E2C2-4F51-9BAE-3F5476477926}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="169">
   <si>
     <t>S No.</t>
   </si>
@@ -520,6 +520,36 @@
   </si>
   <si>
     <t>HSCL</t>
+  </si>
+  <si>
+    <t>TIMETECHNO</t>
+  </si>
+  <si>
+    <t>ICICI BANK</t>
+  </si>
+  <si>
+    <t>JSW</t>
+  </si>
+  <si>
+    <t>ABREL</t>
+  </si>
+  <si>
+    <t>SANSERA</t>
+  </si>
+  <si>
+    <t>PAYTM</t>
+  </si>
+  <si>
+    <t>EMCURE PHARMA</t>
+  </si>
+  <si>
+    <t>LLOYD METALS</t>
+  </si>
+  <si>
+    <t>UNION BANK OF INDIA</t>
+  </si>
+  <si>
+    <t>NAVIN FLUORINE</t>
   </si>
 </sst>
 </file>
@@ -3389,7 +3419,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11702C7E-E6DA-4340-BEE9-A978C9B55E59}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:Q201"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -3456,7 +3485,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3486,7 +3515,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3510,7 +3539,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3540,7 +3569,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3573,7 +3602,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3600,7 +3629,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -3636,7 +3665,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3663,7 +3692,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -3690,7 +3719,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -3717,7 +3746,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -3744,7 +3773,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -3771,7 +3800,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -3798,7 +3827,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3849,7 +3878,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3876,7 +3905,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3906,7 +3935,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
@@ -3930,7 +3959,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
@@ -3960,7 +3989,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
@@ -3984,7 +4013,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
@@ -4008,7 +4037,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
@@ -4035,7 +4064,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
@@ -4068,7 +4097,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
@@ -4098,7 +4127,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
@@ -4134,7 +4163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
@@ -4158,7 +4187,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
@@ -4188,7 +4217,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>27</v>
       </c>
@@ -4220,7 +4249,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>28</v>
       </c>
@@ -4246,7 +4275,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>29</v>
       </c>
@@ -4269,7 +4298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>30</v>
       </c>
@@ -4292,7 +4321,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>31</v>
       </c>
@@ -4315,7 +4344,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>32</v>
       </c>
@@ -4341,7 +4370,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>33</v>
       </c>
@@ -4361,7 +4390,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>34</v>
       </c>
@@ -4381,7 +4410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>35</v>
       </c>
@@ -4404,7 +4433,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>36</v>
       </c>
@@ -4430,7 +4459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>37</v>
       </c>
@@ -4456,7 +4485,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>38</v>
       </c>
@@ -4479,7 +4508,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>39</v>
       </c>
@@ -4499,7 +4528,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>40</v>
       </c>
@@ -4519,7 +4548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>41</v>
       </c>
@@ -4545,7 +4574,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>42</v>
       </c>
@@ -4571,7 +4600,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>43</v>
       </c>
@@ -4591,7 +4620,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>44</v>
       </c>
@@ -4611,7 +4640,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>45</v>
       </c>
@@ -4631,7 +4660,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>46</v>
       </c>
@@ -4651,7 +4680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>47</v>
       </c>
@@ -4671,7 +4700,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>48</v>
       </c>
@@ -4691,7 +4720,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>49</v>
       </c>
@@ -4720,7 +4749,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>50</v>
       </c>
@@ -4746,7 +4775,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>51</v>
       </c>
@@ -4772,7 +4801,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>52</v>
       </c>
@@ -4792,7 +4821,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>53</v>
       </c>
@@ -4815,7 +4844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>54</v>
       </c>
@@ -4835,7 +4864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>55</v>
       </c>
@@ -4855,7 +4884,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>56</v>
       </c>
@@ -4882,7 +4911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>57</v>
       </c>
@@ -4914,7 +4943,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>58</v>
       </c>
@@ -4937,7 +4966,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>59</v>
       </c>
@@ -4963,7 +4992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>60</v>
       </c>
@@ -4983,7 +5012,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>61</v>
       </c>
@@ -5003,7 +5032,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>62</v>
       </c>
@@ -5023,7 +5052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>63</v>
       </c>
@@ -5049,7 +5078,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>64</v>
       </c>
@@ -5075,7 +5104,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>65</v>
       </c>
@@ -5098,7 +5127,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>66</v>
       </c>
@@ -5121,7 +5150,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>67</v>
       </c>
@@ -5141,7 +5170,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>68</v>
       </c>
@@ -5161,7 +5190,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>69</v>
       </c>
@@ -5187,7 +5216,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>70</v>
       </c>
@@ -5207,7 +5236,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>71</v>
       </c>
@@ -5233,7 +5262,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>72</v>
       </c>
@@ -5262,7 +5291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>73</v>
       </c>
@@ -5288,7 +5317,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>74</v>
       </c>
@@ -5308,7 +5337,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>75</v>
       </c>
@@ -5328,7 +5357,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>76</v>
       </c>
@@ -5348,7 +5377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>77</v>
       </c>
@@ -5374,7 +5403,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>78</v>
       </c>
@@ -5406,7 +5435,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>79</v>
       </c>
@@ -5426,7 +5455,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>80</v>
       </c>
@@ -5446,7 +5475,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>81</v>
       </c>
@@ -5472,7 +5501,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>82</v>
       </c>
@@ -5501,7 +5530,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>83</v>
       </c>
@@ -5527,7 +5556,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>84</v>
       </c>
@@ -5550,7 +5579,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>85</v>
       </c>
@@ -5576,7 +5605,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>86</v>
       </c>
@@ -5602,7 +5631,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>87</v>
       </c>
@@ -5622,7 +5651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>88</v>
       </c>
@@ -5642,7 +5671,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>89</v>
       </c>
@@ -5694,7 +5723,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>91</v>
       </c>
@@ -5720,7 +5749,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>92</v>
       </c>
@@ -5740,7 +5769,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>93</v>
       </c>
@@ -5766,7 +5795,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>94</v>
       </c>
@@ -5786,7 +5815,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>95</v>
       </c>
@@ -5812,7 +5841,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>96</v>
       </c>
@@ -5838,7 +5867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>97</v>
       </c>
@@ -5858,7 +5887,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="99" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>98</v>
       </c>
@@ -5872,7 +5901,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="100" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>99</v>
       </c>
@@ -5889,7 +5918,7 @@
         <v>1520</v>
       </c>
     </row>
-    <row r="101" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>100</v>
       </c>
@@ -5906,7 +5935,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="102" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A102">
         <v>101</v>
       </c>
@@ -5926,7 +5955,7 @@
         <v>1035</v>
       </c>
     </row>
-    <row r="103" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>102</v>
       </c>
@@ -5946,7 +5975,7 @@
         <v>968</v>
       </c>
     </row>
-    <row r="104" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>103</v>
       </c>
@@ -5963,7 +5992,7 @@
         <v>2750</v>
       </c>
     </row>
-    <row r="105" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A105">
         <v>104</v>
       </c>
@@ -5977,7 +6006,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="106" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>105</v>
       </c>
@@ -5991,7 +6020,7 @@
         <v>802</v>
       </c>
     </row>
-    <row r="107" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A107">
         <v>106</v>
       </c>
@@ -6011,7 +6040,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="108" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A108">
         <v>107</v>
       </c>
@@ -6028,7 +6057,7 @@
         <v>1940</v>
       </c>
     </row>
-    <row r="109" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>108</v>
       </c>
@@ -6045,7 +6074,7 @@
         <v>1780</v>
       </c>
     </row>
-    <row r="110" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>109</v>
       </c>
@@ -6059,7 +6088,7 @@
         <v>976</v>
       </c>
     </row>
-    <row r="111" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>110</v>
       </c>
@@ -6073,7 +6102,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="112" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>111</v>
       </c>
@@ -6093,7 +6122,7 @@
         <v>1540</v>
       </c>
     </row>
-    <row r="113" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>112</v>
       </c>
@@ -6113,7 +6142,7 @@
         <v>1331</v>
       </c>
     </row>
-    <row r="114" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>113</v>
       </c>
@@ -6127,7 +6156,7 @@
         <v>1018</v>
       </c>
     </row>
-    <row r="115" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>114</v>
       </c>
@@ -6144,7 +6173,7 @@
         <v>950</v>
       </c>
     </row>
-    <row r="116" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>115</v>
       </c>
@@ -6158,7 +6187,7 @@
         <v>1027</v>
       </c>
     </row>
-    <row r="117" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>116</v>
       </c>
@@ -6172,7 +6201,7 @@
         <v>1360</v>
       </c>
     </row>
-    <row r="118" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>117</v>
       </c>
@@ -6192,7 +6221,7 @@
         <v>1810</v>
       </c>
     </row>
-    <row r="119" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>118</v>
       </c>
@@ -6209,7 +6238,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="120" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>119</v>
       </c>
@@ -6229,7 +6258,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="121" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>120</v>
       </c>
@@ -6243,7 +6272,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="122" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>121</v>
       </c>
@@ -6257,7 +6286,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="123" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>122</v>
       </c>
@@ -6274,7 +6303,7 @@
         <v>5250</v>
       </c>
     </row>
-    <row r="124" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>123</v>
       </c>
@@ -6288,7 +6317,7 @@
         <v>2246</v>
       </c>
     </row>
-    <row r="125" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>124</v>
       </c>
@@ -6302,7 +6331,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="126" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>125</v>
       </c>
@@ -6322,7 +6351,7 @@
         <v>3130</v>
       </c>
     </row>
-    <row r="127" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>126</v>
       </c>
@@ -6343,7 +6372,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="128" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>127</v>
       </c>
@@ -6357,7 +6386,7 @@
         <v>1516</v>
       </c>
     </row>
-    <row r="129" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A129">
         <v>128</v>
       </c>
@@ -6371,7 +6400,7 @@
         <v>1110</v>
       </c>
     </row>
-    <row r="130" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A130">
         <v>129</v>
       </c>
@@ -6388,7 +6417,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="131" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A131">
         <v>130</v>
       </c>
@@ -6402,7 +6431,7 @@
         <v>1785</v>
       </c>
     </row>
-    <row r="132" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A132">
         <v>131</v>
       </c>
@@ -6425,7 +6454,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="133" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A133">
         <v>132</v>
       </c>
@@ -6442,7 +6471,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="134" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A134">
         <v>133</v>
       </c>
@@ -6459,7 +6488,7 @@
         <v>1406</v>
       </c>
     </row>
-    <row r="135" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A135">
         <v>134</v>
       </c>
@@ -6473,7 +6502,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="136" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A136">
         <v>135</v>
       </c>
@@ -6496,7 +6525,7 @@
         <v>1150</v>
       </c>
     </row>
-    <row r="137" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A137">
         <v>136</v>
       </c>
@@ -6519,7 +6548,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="138" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A138">
         <v>137</v>
       </c>
@@ -6539,7 +6568,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="139" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A139">
         <v>138</v>
       </c>
@@ -6559,7 +6588,7 @@
         <v>16100</v>
       </c>
     </row>
-    <row r="140" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A140">
         <v>139</v>
       </c>
@@ -6576,7 +6605,7 @@
         <v>1507</v>
       </c>
     </row>
-    <row r="141" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A141">
         <v>140</v>
       </c>
@@ -6590,7 +6619,7 @@
         <v>1954</v>
       </c>
     </row>
-    <row r="142" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A142">
         <v>141</v>
       </c>
@@ -6613,7 +6642,7 @@
         <v>3290</v>
       </c>
     </row>
-    <row r="143" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A143">
         <v>142</v>
       </c>
@@ -6636,7 +6665,7 @@
         <v>1380</v>
       </c>
     </row>
-    <row r="144" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A144">
         <v>143</v>
       </c>
@@ -6650,7 +6679,7 @@
         <v>46216</v>
       </c>
     </row>
-    <row r="145" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A145">
         <v>144</v>
       </c>
@@ -6661,7 +6690,7 @@
         <v>46216</v>
       </c>
     </row>
-    <row r="146" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A146">
         <v>145</v>
       </c>
@@ -6678,7 +6707,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="147" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A147">
         <v>146</v>
       </c>
@@ -6695,7 +6724,7 @@
         <v>1025</v>
       </c>
     </row>
-    <row r="148" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A148">
         <v>147</v>
       </c>
@@ -6718,7 +6747,7 @@
         <v>968</v>
       </c>
     </row>
-    <row r="149" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A149">
         <v>148</v>
       </c>
@@ -6738,7 +6767,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="150" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A150">
         <v>149</v>
       </c>
@@ -6755,7 +6784,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="151" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A151">
         <v>150</v>
       </c>
@@ -6769,7 +6798,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="152" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A152">
         <v>151</v>
       </c>
@@ -6786,7 +6815,7 @@
         <v>3800</v>
       </c>
     </row>
-    <row r="153" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A153">
         <v>152</v>
       </c>
@@ -6803,7 +6832,7 @@
         <v>1450</v>
       </c>
     </row>
-    <row r="154" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A154">
         <v>153</v>
       </c>
@@ -6823,7 +6852,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="155" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A155">
         <v>154</v>
       </c>
@@ -6843,7 +6872,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="156" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A156">
         <v>155</v>
       </c>
@@ -6860,7 +6889,7 @@
         <v>1604</v>
       </c>
     </row>
-    <row r="157" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A157">
         <v>156</v>
       </c>
@@ -6877,7 +6906,7 @@
         <v>1826</v>
       </c>
     </row>
-    <row r="158" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A158">
         <v>157</v>
       </c>
@@ -6897,7 +6926,7 @@
         <v>1790</v>
       </c>
     </row>
-    <row r="159" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A159">
         <v>158</v>
       </c>
@@ -6920,7 +6949,7 @@
         <v>1800</v>
       </c>
     </row>
-    <row r="160" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A160">
         <v>159</v>
       </c>
@@ -6937,7 +6966,7 @@
         <v>7203</v>
       </c>
     </row>
-    <row r="161" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A161">
         <v>160</v>
       </c>
@@ -6954,7 +6983,7 @@
         <v>4133</v>
       </c>
     </row>
-    <row r="162" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A162">
         <v>161</v>
       </c>
@@ -6994,7 +7023,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="164" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A164">
         <v>163</v>
       </c>
@@ -7017,13 +7046,16 @@
         <v>1035</v>
       </c>
     </row>
-    <row r="165" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A165">
         <v>164</v>
       </c>
       <c r="B165" t="s">
         <v>153</v>
       </c>
+      <c r="D165" s="1">
+        <v>46220</v>
+      </c>
       <c r="E165">
         <v>350</v>
       </c>
@@ -7031,13 +7063,16 @@
         <v>420</v>
       </c>
     </row>
-    <row r="166" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A166">
         <v>165</v>
       </c>
       <c r="B166" t="s">
         <v>154</v>
       </c>
+      <c r="D166" s="1">
+        <v>46220</v>
+      </c>
       <c r="E166">
         <v>1510</v>
       </c>
@@ -7045,13 +7080,16 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="167" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A167">
         <v>166</v>
       </c>
       <c r="B167" t="s">
         <v>155</v>
       </c>
+      <c r="D167" s="1">
+        <v>46220</v>
+      </c>
       <c r="E167">
         <v>2185</v>
       </c>
@@ -7059,29 +7097,38 @@
         <v>2620</v>
       </c>
     </row>
-    <row r="168" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A168">
         <v>167</v>
       </c>
       <c r="B168" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="169" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="D168" s="1">
+        <v>46220</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A169">
         <v>168</v>
       </c>
       <c r="B169" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="170" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="D169" s="1">
+        <v>46220</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A170">
         <v>169</v>
       </c>
       <c r="B170" s="4" t="s">
         <v>158</v>
       </c>
+      <c r="D170" s="1">
+        <v>46220</v>
+      </c>
       <c r="E170">
         <v>725</v>
       </c>
@@ -7092,169 +7139,301 @@
         <v>695</v>
       </c>
     </row>
-    <row r="171" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A171">
         <v>170</v>
       </c>
-    </row>
-    <row r="172" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="B171" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C171" t="s">
+        <v>124</v>
+      </c>
+      <c r="D171" s="1">
+        <v>46223</v>
+      </c>
+      <c r="E171">
+        <v>435</v>
+      </c>
+      <c r="F171">
+        <v>475</v>
+      </c>
+      <c r="G171">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A172">
         <v>171</v>
       </c>
-    </row>
-    <row r="173" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="B172" t="s">
+        <v>139</v>
+      </c>
+      <c r="D172" s="1">
+        <v>46223</v>
+      </c>
+      <c r="E172">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A173">
         <v>172</v>
       </c>
-    </row>
-    <row r="174" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="B173" t="s">
+        <v>159</v>
+      </c>
+      <c r="D173" s="1">
+        <v>46223</v>
+      </c>
+      <c r="E173">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A174">
         <v>173</v>
       </c>
-    </row>
-    <row r="175" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="B174" t="s">
+        <v>160</v>
+      </c>
+      <c r="D174" s="1">
+        <v>46223</v>
+      </c>
+      <c r="E174">
+        <v>14444</v>
+      </c>
+      <c r="F174">
+        <v>1750</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A175">
         <v>174</v>
       </c>
-    </row>
-    <row r="176" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="B175" t="s">
+        <v>161</v>
+      </c>
+      <c r="D175" s="1">
+        <v>46223</v>
+      </c>
+      <c r="E175">
+        <v>1237</v>
+      </c>
+      <c r="F175">
+        <v>1470</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A176">
         <v>175</v>
       </c>
-    </row>
-    <row r="177" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+      <c r="B176" t="s">
+        <v>162</v>
+      </c>
+      <c r="D176" s="1">
+        <v>46223</v>
+      </c>
+      <c r="E176">
+        <v>1412</v>
+      </c>
+      <c r="F176">
+        <v>1586</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A177">
         <v>176</v>
       </c>
-    </row>
-    <row r="178" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+      <c r="B177" t="s">
+        <v>163</v>
+      </c>
+      <c r="C177" t="s">
+        <v>124</v>
+      </c>
+      <c r="D177" s="1">
+        <v>46223</v>
+      </c>
+      <c r="E177">
+        <v>3388</v>
+      </c>
+      <c r="F177">
+        <v>3684</v>
+      </c>
+      <c r="G177">
+        <v>3240</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A178">
         <v>177</v>
       </c>
-    </row>
-    <row r="179" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+      <c r="B178" t="s">
+        <v>164</v>
+      </c>
+      <c r="D178" s="1">
+        <v>46224</v>
+      </c>
+      <c r="E178">
+        <v>1348</v>
+      </c>
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A179">
         <v>178</v>
       </c>
-    </row>
-    <row r="180" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+      <c r="B179" t="s">
+        <v>165</v>
+      </c>
+      <c r="D179" s="1">
+        <v>46224</v>
+      </c>
+      <c r="E179">
+        <v>1862</v>
+      </c>
+      <c r="F179">
+        <v>2260</v>
+      </c>
+    </row>
+    <row r="180" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A180">
         <v>179</v>
       </c>
-    </row>
-    <row r="181" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+      <c r="B180" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="D180" s="1">
+        <v>46224</v>
+      </c>
+      <c r="E180">
+        <v>1908</v>
+      </c>
+      <c r="F180">
+        <v>2070</v>
+      </c>
+      <c r="G180">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="181" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A181">
         <v>180</v>
       </c>
-    </row>
-    <row r="182" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+      <c r="B181" t="s">
+        <v>167</v>
+      </c>
+      <c r="D181" s="1">
+        <v>46224</v>
+      </c>
+    </row>
+    <row r="182" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A182">
         <v>181</v>
       </c>
-    </row>
-    <row r="183" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+      <c r="B182" t="s">
+        <v>168</v>
+      </c>
+      <c r="D182" s="1">
+        <v>46224</v>
+      </c>
+    </row>
+    <row r="183" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A183">
         <v>182</v>
       </c>
     </row>
-    <row r="184" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A184">
         <v>183</v>
       </c>
     </row>
-    <row r="185" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A185">
         <v>184</v>
       </c>
     </row>
-    <row r="186" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A186">
         <v>185</v>
       </c>
     </row>
-    <row r="187" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A187">
         <v>186</v>
       </c>
     </row>
-    <row r="188" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A188">
         <v>187</v>
       </c>
     </row>
-    <row r="189" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A189">
         <v>188</v>
       </c>
     </row>
-    <row r="190" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A190">
         <v>189</v>
       </c>
     </row>
-    <row r="191" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A191">
         <v>190</v>
       </c>
     </row>
-    <row r="192" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A192">
         <v>191</v>
       </c>
     </row>
-    <row r="193" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A193">
         <v>192</v>
       </c>
     </row>
-    <row r="194" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A194">
         <v>193</v>
       </c>
     </row>
-    <row r="195" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A195">
         <v>194</v>
       </c>
     </row>
-    <row r="196" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A196">
         <v>195</v>
       </c>
     </row>
-    <row r="197" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A197">
         <v>196</v>
       </c>
     </row>
-    <row r="198" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A198">
         <v>197</v>
       </c>
     </row>
-    <row r="199" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A199">
         <v>198</v>
       </c>
     </row>
-    <row r="200" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A200">
         <v>199</v>
       </c>
     </row>
-    <row r="201" spans="1:1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A201">
         <v>200</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L201" xr:uid="{11702C7E-E6DA-4340-BEE9-A978C9B55E59}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="GROWW"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:L201" xr:uid="{11702C7E-E6DA-4340-BEE9-A978C9B55E59}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>

</xml_diff>